<commit_message>
Costo y Margen en Excel
</commit_message>
<xml_diff>
--- a/docs/Costos_BZM_PDG.xlsx
+++ b/docs/Costos_BZM_PDG.xlsx
@@ -1,21 +1,25 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\e3031434\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/098a8ea1b880659c/Documents/GitHub/Eaton/docs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{7DAE8A73-595C-4E0D-ADD0-D42089A262DB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="27" documentId="8_{7DAE8A73-595C-4E0D-ADD0-D42089A262DB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{36A894CB-4307-4FC0-84B1-FE4310788745}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{9590C155-5574-4B57-8D25-D452FF3E0533}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" activeTab="1" xr2:uid="{9590C155-5574-4B57-8D25-D452FF3E0533}"/>
   </bookViews>
   <sheets>
     <sheet name="BZM" sheetId="1" r:id="rId1"/>
     <sheet name="PDG" sheetId="2" r:id="rId2"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">BZM!$A$1:$D$45</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">PDG!$A$1:$D$221</definedName>
+  </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -2446,16 +2450,17 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6CE20DDE-3F02-4F40-B514-62B99779A301}">
+  <sheetPr filterMode="1"/>
   <dimension ref="A1:D45"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="15.42578125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="15.44140625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="15" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="42.7109375" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="11.42578125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="42.6640625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="11.44140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -2469,7 +2474,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A2">
         <v>111554</v>
       </c>
@@ -2483,7 +2488,7 @@
         <v>384.24</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A3">
         <v>111555</v>
       </c>
@@ -2497,7 +2502,7 @@
         <v>384.24</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A4">
         <v>111557</v>
       </c>
@@ -2511,7 +2516,7 @@
         <v>380.71</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A5">
         <v>111558</v>
       </c>
@@ -2525,7 +2530,7 @@
         <v>582.79</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A6">
         <v>111560</v>
       </c>
@@ -2539,7 +2544,7 @@
         <v>366.81</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A7">
         <v>111561</v>
       </c>
@@ -2553,7 +2558,7 @@
         <v>366.81</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A8">
         <v>111563</v>
       </c>
@@ -2567,7 +2572,7 @@
         <v>371.17</v>
       </c>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A9">
         <v>111564</v>
       </c>
@@ -2581,7 +2586,7 @@
         <v>371.17</v>
       </c>
     </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A10">
         <v>111566</v>
       </c>
@@ -2595,7 +2600,7 @@
         <v>374.08</v>
       </c>
     </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A11">
         <v>111567</v>
       </c>
@@ -2609,7 +2614,7 @@
         <v>374.08</v>
       </c>
     </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A12">
         <v>111569</v>
       </c>
@@ -2623,7 +2628,7 @@
         <v>361.83</v>
       </c>
     </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A13">
         <v>111570</v>
       </c>
@@ -2637,7 +2642,7 @@
         <v>361.83</v>
       </c>
     </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A14">
         <v>111572</v>
       </c>
@@ -2651,7 +2656,7 @@
         <v>359.76</v>
       </c>
     </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A15">
         <v>111573</v>
       </c>
@@ -2665,7 +2670,7 @@
         <v>359.76</v>
       </c>
     </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A16">
         <v>111575</v>
       </c>
@@ -2679,7 +2684,7 @@
         <v>371.38</v>
       </c>
     </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A17">
         <v>111576</v>
       </c>
@@ -2693,7 +2698,7 @@
         <v>371.38</v>
       </c>
     </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A18">
         <v>111578</v>
       </c>
@@ -2707,7 +2712,7 @@
         <v>375.32</v>
       </c>
     </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A19">
         <v>111579</v>
       </c>
@@ -2721,7 +2726,7 @@
         <v>539.42999999999995</v>
       </c>
     </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A20">
         <v>116973</v>
       </c>
@@ -2735,7 +2740,7 @@
         <v>1360.45</v>
       </c>
     </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A21">
         <v>116974</v>
       </c>
@@ -2749,7 +2754,7 @@
         <v>1545.18</v>
       </c>
     </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A22">
         <v>116975</v>
       </c>
@@ -2763,7 +2768,7 @@
         <v>1614.84</v>
       </c>
     </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A23">
         <v>119735</v>
       </c>
@@ -2777,7 +2782,7 @@
         <v>1268.8599999999999</v>
       </c>
     </row>
-    <row r="24" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A24">
         <v>121804</v>
       </c>
@@ -2791,7 +2796,7 @@
         <v>1170.9100000000001</v>
       </c>
     </row>
-    <row r="25" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A25">
         <v>121805</v>
       </c>
@@ -2805,7 +2810,7 @@
         <v>1192.6600000000001</v>
       </c>
     </row>
-    <row r="26" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A26">
         <v>121806</v>
       </c>
@@ -2819,7 +2824,7 @@
         <v>1425.3</v>
       </c>
     </row>
-    <row r="27" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A27">
         <v>121807</v>
       </c>
@@ -2833,7 +2838,7 @@
         <v>1536.52</v>
       </c>
     </row>
-    <row r="28" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A28">
         <v>131276</v>
       </c>
@@ -2847,7 +2852,7 @@
         <v>609.14</v>
       </c>
     </row>
-    <row r="29" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A29">
         <v>131277</v>
       </c>
@@ -2861,7 +2866,7 @@
         <v>570.97</v>
       </c>
     </row>
-    <row r="30" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A30">
         <v>131278</v>
       </c>
@@ -2875,7 +2880,7 @@
         <v>580.92999999999995</v>
       </c>
     </row>
-    <row r="31" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A31">
         <v>131279</v>
       </c>
@@ -2889,7 +2894,7 @@
         <v>387.35</v>
       </c>
     </row>
-    <row r="32" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A32">
         <v>131280</v>
       </c>
@@ -2903,7 +2908,7 @@
         <v>712.88</v>
       </c>
     </row>
-    <row r="33" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A33">
         <v>131281</v>
       </c>
@@ -2917,7 +2922,7 @@
         <v>1243.5999999999999</v>
       </c>
     </row>
-    <row r="34" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A34">
         <v>158276</v>
       </c>
@@ -2931,7 +2936,7 @@
         <v>1400.45</v>
       </c>
     </row>
-    <row r="35" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A35">
         <v>158277</v>
       </c>
@@ -2945,7 +2950,7 @@
         <v>1400.45</v>
       </c>
     </row>
-    <row r="36" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A36">
         <v>158278</v>
       </c>
@@ -2959,7 +2964,7 @@
         <v>1401.9</v>
       </c>
     </row>
-    <row r="37" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A37">
         <v>158279</v>
       </c>
@@ -2973,7 +2978,7 @@
         <v>1400.45</v>
       </c>
     </row>
-    <row r="38" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A38">
         <v>158280</v>
       </c>
@@ -2987,7 +2992,7 @@
         <v>1834.28</v>
       </c>
     </row>
-    <row r="39" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A39">
         <v>158281</v>
       </c>
@@ -3001,7 +3006,7 @@
         <v>1400.45</v>
       </c>
     </row>
-    <row r="40" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A40">
         <v>158282</v>
       </c>
@@ -3015,7 +3020,7 @@
         <v>1400.45</v>
       </c>
     </row>
-    <row r="41" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A41">
         <v>158283</v>
       </c>
@@ -3029,7 +3034,7 @@
         <v>1400.45</v>
       </c>
     </row>
-    <row r="42" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A42">
         <v>158284</v>
       </c>
@@ -3043,7 +3048,7 @@
         <v>1400.45</v>
       </c>
     </row>
-    <row r="43" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A43">
         <v>158285</v>
       </c>
@@ -3057,7 +3062,7 @@
         <v>2225.7800000000002</v>
       </c>
     </row>
-    <row r="44" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A44">
         <v>158286</v>
       </c>
@@ -3071,7 +3076,7 @@
         <v>2225.7800000000002</v>
       </c>
     </row>
-    <row r="45" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A45">
         <v>158287</v>
       </c>
@@ -3086,21 +3091,32 @@
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="A1:D45" xr:uid="{6CE20DDE-3F02-4F40-B514-62B99779A301}">
+    <filterColumn colId="2">
+      <filters>
+        <filter val="BZMN3-A250-AP"/>
+        <filter val="BZMN3-A320-AP"/>
+        <filter val="BZMN3-A350-AP"/>
+        <filter val="BZMN3-A400-AP"/>
+      </filters>
+    </filterColumn>
+  </autoFilter>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7946CC59-6F99-4531-BC40-6D94404CB3C2}">
+  <sheetPr filterMode="1"/>
   <dimension ref="A1:D221"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="2" width="17.85546875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="39.85546875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="11.42578125" bestFit="1" customWidth="1"/>
+    <col min="1" max="2" width="17.88671875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="39.88671875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="11.44140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -3114,7 +3130,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>48</v>
       </c>
@@ -3128,7 +3144,7 @@
         <v>2185.9499999999998</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>49</v>
       </c>
@@ -3142,7 +3158,7 @@
         <v>2256.69</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>52</v>
       </c>
@@ -3156,7 +3172,7 @@
         <v>2006.69</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>54</v>
       </c>
@@ -3170,7 +3186,7 @@
         <v>2006.69</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>56</v>
       </c>
@@ -3184,7 +3200,7 @@
         <v>1911.04</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>58</v>
       </c>
@@ -3198,7 +3214,7 @@
         <v>1925.77</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>60</v>
       </c>
@@ -3212,7 +3228,7 @@
         <v>1930.34</v>
       </c>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>62</v>
       </c>
@@ -3226,7 +3242,7 @@
         <v>1934.9</v>
       </c>
     </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>64</v>
       </c>
@@ -3240,7 +3256,7 @@
         <v>1931.79</v>
       </c>
     </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>66</v>
       </c>
@@ -3254,7 +3270,7 @@
         <v>1910.84</v>
       </c>
     </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>68</v>
       </c>
@@ -3268,7 +3284,7 @@
         <v>1978.47</v>
       </c>
     </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>70</v>
       </c>
@@ -3282,7 +3298,7 @@
         <v>2326.41</v>
       </c>
     </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>72</v>
       </c>
@@ -3296,7 +3312,7 @@
         <v>2466.66</v>
       </c>
     </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>74</v>
       </c>
@@ -3310,7 +3326,7 @@
         <v>2451.31</v>
       </c>
     </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
         <v>76</v>
       </c>
@@ -3324,7 +3340,7 @@
         <v>2257.3200000000002</v>
       </c>
     </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
         <v>78</v>
       </c>
@@ -3338,7 +3354,7 @@
         <v>2246.11</v>
       </c>
     </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
         <v>80</v>
       </c>
@@ -3352,7 +3368,7 @@
         <v>1930.34</v>
       </c>
     </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
         <v>81</v>
       </c>
@@ -3366,7 +3382,7 @@
         <v>2282.63</v>
       </c>
     </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
         <v>83</v>
       </c>
@@ -3380,7 +3396,7 @@
         <v>2278.89</v>
       </c>
     </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
         <v>88</v>
       </c>
@@ -3394,7 +3410,7 @@
         <v>969.53</v>
       </c>
     </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
         <v>90</v>
       </c>
@@ -3408,7 +3424,7 @@
         <v>953.76</v>
       </c>
     </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
         <v>92</v>
       </c>
@@ -3422,7 +3438,7 @@
         <v>948.16</v>
       </c>
     </row>
-    <row r="24" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
         <v>94</v>
       </c>
@@ -3436,7 +3452,7 @@
         <v>923.47</v>
       </c>
     </row>
-    <row r="25" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
         <v>96</v>
       </c>
@@ -3450,7 +3466,7 @@
         <v>947.12</v>
       </c>
     </row>
-    <row r="26" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
         <v>98</v>
       </c>
@@ -3464,7 +3480,7 @@
         <v>1346.92</v>
       </c>
     </row>
-    <row r="27" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
         <v>100</v>
       </c>
@@ -3478,7 +3494,7 @@
         <v>1313.31</v>
       </c>
     </row>
-    <row r="28" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
         <v>102</v>
       </c>
@@ -3492,7 +3508,7 @@
         <v>1328.66</v>
       </c>
     </row>
-    <row r="29" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
         <v>104</v>
       </c>
@@ -3506,7 +3522,7 @@
         <v>1330.32</v>
       </c>
     </row>
-    <row r="30" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
         <v>106</v>
       </c>
@@ -3520,7 +3536,7 @@
         <v>1329.08</v>
       </c>
     </row>
-    <row r="31" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
         <v>108</v>
       </c>
@@ -3534,7 +3550,7 @@
         <v>1389.04</v>
       </c>
     </row>
-    <row r="32" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
         <v>110</v>
       </c>
@@ -3548,7 +3564,7 @@
         <v>1412.28</v>
       </c>
     </row>
-    <row r="33" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
         <v>112</v>
       </c>
@@ -3562,7 +3578,7 @@
         <v>1405.84</v>
       </c>
     </row>
-    <row r="34" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A34" t="s">
         <v>114</v>
       </c>
@@ -3576,7 +3592,7 @@
         <v>1407.71</v>
       </c>
     </row>
-    <row r="35" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A35" t="s">
         <v>116</v>
       </c>
@@ -3590,7 +3606,7 @@
         <v>1481.99</v>
       </c>
     </row>
-    <row r="36" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A36" t="s">
         <v>118</v>
       </c>
@@ -3604,7 +3620,7 @@
         <v>1481.99</v>
       </c>
     </row>
-    <row r="37" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A37" t="s">
         <v>120</v>
       </c>
@@ -3618,7 +3634,7 @@
         <v>1528.67</v>
       </c>
     </row>
-    <row r="38" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A38" t="s">
         <v>122</v>
       </c>
@@ -3632,7 +3648,7 @@
         <v>1527.22</v>
       </c>
     </row>
-    <row r="39" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A39" t="s">
         <v>124</v>
       </c>
@@ -3646,7 +3662,7 @@
         <v>1618.09</v>
       </c>
     </row>
-    <row r="40" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A40" t="s">
         <v>126</v>
       </c>
@@ -3660,7 +3676,7 @@
         <v>1346.92</v>
       </c>
     </row>
-    <row r="41" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A41" t="s">
         <v>128</v>
       </c>
@@ -3674,7 +3690,7 @@
         <v>1313.31</v>
       </c>
     </row>
-    <row r="42" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A42" t="s">
         <v>130</v>
       </c>
@@ -3688,7 +3704,7 @@
         <v>1328.66</v>
       </c>
     </row>
-    <row r="43" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A43" t="s">
         <v>132</v>
       </c>
@@ -3702,7 +3718,7 @@
         <v>1330.32</v>
       </c>
     </row>
-    <row r="44" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A44" t="s">
         <v>134</v>
       </c>
@@ -3716,7 +3732,7 @@
         <v>1329.08</v>
       </c>
     </row>
-    <row r="45" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A45" t="s">
         <v>136</v>
       </c>
@@ -3730,7 +3746,7 @@
         <v>1389.04</v>
       </c>
     </row>
-    <row r="46" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A46" t="s">
         <v>138</v>
       </c>
@@ -3744,7 +3760,7 @@
         <v>1412.28</v>
       </c>
     </row>
-    <row r="47" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A47" t="s">
         <v>140</v>
       </c>
@@ -3758,7 +3774,7 @@
         <v>1407.71</v>
       </c>
     </row>
-    <row r="48" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A48" t="s">
         <v>142</v>
       </c>
@@ -3772,7 +3788,7 @@
         <v>1481.99</v>
       </c>
     </row>
-    <row r="49" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A49" t="s">
         <v>144</v>
       </c>
@@ -3786,7 +3802,7 @@
         <v>1481.99</v>
       </c>
     </row>
-    <row r="50" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A50" t="s">
         <v>146</v>
       </c>
@@ -3800,7 +3816,7 @@
         <v>1527.22</v>
       </c>
     </row>
-    <row r="51" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A51" t="s">
         <v>148</v>
       </c>
@@ -3814,7 +3830,7 @@
         <v>1618.09</v>
       </c>
     </row>
-    <row r="52" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A52" t="s">
         <v>150</v>
       </c>
@@ -3828,7 +3844,7 @@
         <v>1346.92</v>
       </c>
     </row>
-    <row r="53" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A53" t="s">
         <v>152</v>
       </c>
@@ -3842,7 +3858,7 @@
         <v>1313.31</v>
       </c>
     </row>
-    <row r="54" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A54" t="s">
         <v>154</v>
       </c>
@@ -3856,7 +3872,7 @@
         <v>1328.66</v>
       </c>
     </row>
-    <row r="55" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A55" t="s">
         <v>156</v>
       </c>
@@ -3870,7 +3886,7 @@
         <v>1330.32</v>
       </c>
     </row>
-    <row r="56" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A56" t="s">
         <v>158</v>
       </c>
@@ -3884,7 +3900,7 @@
         <v>1329.08</v>
       </c>
     </row>
-    <row r="57" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A57" t="s">
         <v>160</v>
       </c>
@@ -3898,7 +3914,7 @@
         <v>1412.28</v>
       </c>
     </row>
-    <row r="58" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A58" t="s">
         <v>162</v>
       </c>
@@ -3912,7 +3928,7 @@
         <v>1407.71</v>
       </c>
     </row>
-    <row r="59" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A59" t="s">
         <v>164</v>
       </c>
@@ -3926,7 +3942,7 @@
         <v>1481.99</v>
       </c>
     </row>
-    <row r="60" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A60" t="s">
         <v>166</v>
       </c>
@@ -3940,7 +3956,7 @@
         <v>1481.99</v>
       </c>
     </row>
-    <row r="61" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A61" t="s">
         <v>168</v>
       </c>
@@ -3954,7 +3970,7 @@
         <v>1324.1</v>
       </c>
     </row>
-    <row r="62" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A62" t="s">
         <v>170</v>
       </c>
@@ -3968,7 +3984,7 @@
         <v>1278.25</v>
       </c>
     </row>
-    <row r="63" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A63" t="s">
         <v>172</v>
       </c>
@@ -3982,7 +3998,7 @@
         <v>1288.21</v>
       </c>
     </row>
-    <row r="64" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A64" t="s">
         <v>174</v>
       </c>
@@ -3996,7 +4012,7 @@
         <v>1286.55</v>
       </c>
     </row>
-    <row r="65" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A65" t="s">
         <v>176</v>
       </c>
@@ -4010,7 +4026,7 @@
         <v>1285.0899999999999</v>
       </c>
     </row>
-    <row r="66" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A66" t="s">
         <v>178</v>
       </c>
@@ -4024,7 +4040,7 @@
         <v>1401.49</v>
       </c>
     </row>
-    <row r="67" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A67" t="s">
         <v>180</v>
       </c>
@@ -4038,7 +4054,7 @@
         <v>1409.37</v>
       </c>
     </row>
-    <row r="68" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A68" t="s">
         <v>182</v>
       </c>
@@ -4052,7 +4068,7 @@
         <v>1399.62</v>
       </c>
     </row>
-    <row r="69" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A69" t="s">
         <v>184</v>
       </c>
@@ -4066,7 +4082,7 @@
         <v>1401.28</v>
       </c>
     </row>
-    <row r="70" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A70" t="s">
         <v>186</v>
       </c>
@@ -4080,7 +4096,7 @@
         <v>1568.92</v>
       </c>
     </row>
-    <row r="71" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A71" t="s">
         <v>188</v>
       </c>
@@ -4094,7 +4110,7 @@
         <v>1606.89</v>
       </c>
     </row>
-    <row r="72" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A72" t="s">
         <v>190</v>
       </c>
@@ -4108,7 +4124,7 @@
         <v>1629.71</v>
       </c>
     </row>
-    <row r="73" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A73" t="s">
         <v>192</v>
       </c>
@@ -4122,7 +4138,7 @@
         <v>1627.84</v>
       </c>
     </row>
-    <row r="74" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A74" t="s">
         <v>194</v>
       </c>
@@ -4136,7 +4152,7 @@
         <v>1771.62</v>
       </c>
     </row>
-    <row r="75" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A75" t="s">
         <v>196</v>
       </c>
@@ -4150,7 +4166,7 @@
         <v>1324.1</v>
       </c>
     </row>
-    <row r="76" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A76" t="s">
         <v>198</v>
       </c>
@@ -4164,7 +4180,7 @@
         <v>1278.25</v>
       </c>
     </row>
-    <row r="77" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A77" t="s">
         <v>256</v>
       </c>
@@ -4178,7 +4194,7 @@
         <v>1288.21</v>
       </c>
     </row>
-    <row r="78" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A78" t="s">
         <v>258</v>
       </c>
@@ -4192,7 +4208,7 @@
         <v>1286.55</v>
       </c>
     </row>
-    <row r="79" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A79" t="s">
         <v>260</v>
       </c>
@@ -4206,7 +4222,7 @@
         <v>1285.0899999999999</v>
       </c>
     </row>
-    <row r="80" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A80" t="s">
         <v>262</v>
       </c>
@@ -4220,7 +4236,7 @@
         <v>5223.16</v>
       </c>
     </row>
-    <row r="81" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A81" t="s">
         <v>264</v>
       </c>
@@ -4234,7 +4250,7 @@
         <v>5346.6</v>
       </c>
     </row>
-    <row r="82" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A82" t="s">
         <v>266</v>
       </c>
@@ -4248,7 +4264,7 @@
         <v>1401.49</v>
       </c>
     </row>
-    <row r="83" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A83" t="s">
         <v>268</v>
       </c>
@@ -4262,7 +4278,7 @@
         <v>1409.37</v>
       </c>
     </row>
-    <row r="84" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A84" t="s">
         <v>270</v>
       </c>
@@ -4276,7 +4292,7 @@
         <v>1399.62</v>
       </c>
     </row>
-    <row r="85" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="85" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A85" t="s">
         <v>272</v>
       </c>
@@ -4290,7 +4306,7 @@
         <v>5223.16</v>
       </c>
     </row>
-    <row r="86" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="86" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A86" t="s">
         <v>274</v>
       </c>
@@ -4304,7 +4320,7 @@
         <v>5346.6</v>
       </c>
     </row>
-    <row r="87" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="87" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A87" t="s">
         <v>276</v>
       </c>
@@ -4318,7 +4334,7 @@
         <v>1401.28</v>
       </c>
     </row>
-    <row r="88" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="88" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A88" t="s">
         <v>278</v>
       </c>
@@ -4332,7 +4348,7 @@
         <v>1568.92</v>
       </c>
     </row>
-    <row r="89" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="89" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A89" t="s">
         <v>280</v>
       </c>
@@ -4346,7 +4362,7 @@
         <v>5328.35</v>
       </c>
     </row>
-    <row r="90" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="90" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A90" t="s">
         <v>282</v>
       </c>
@@ -4360,7 +4376,7 @@
         <v>5451.59</v>
       </c>
     </row>
-    <row r="91" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="91" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A91" t="s">
         <v>284</v>
       </c>
@@ -4374,7 +4390,7 @@
         <v>1606.89</v>
       </c>
     </row>
-    <row r="92" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="92" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A92" t="s">
         <v>286</v>
       </c>
@@ -4388,7 +4404,7 @@
         <v>1629.71</v>
       </c>
     </row>
-    <row r="93" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="93" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A93" t="s">
         <v>288</v>
       </c>
@@ -4402,7 +4418,7 @@
         <v>1627.84</v>
       </c>
     </row>
-    <row r="94" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="94" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A94" t="s">
         <v>290</v>
       </c>
@@ -4416,7 +4432,7 @@
         <v>5387.06</v>
       </c>
     </row>
-    <row r="95" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="95" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A95" t="s">
         <v>292</v>
       </c>
@@ -4430,7 +4446,7 @@
         <v>5510.72</v>
       </c>
     </row>
-    <row r="96" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="96" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A96" t="s">
         <v>294</v>
       </c>
@@ -4444,7 +4460,7 @@
         <v>1771.62</v>
       </c>
     </row>
-    <row r="97" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="97" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A97" t="s">
         <v>296</v>
       </c>
@@ -4458,7 +4474,7 @@
         <v>2085.11</v>
       </c>
     </row>
-    <row r="98" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="98" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A98" t="s">
         <v>298</v>
       </c>
@@ -4472,7 +4488,7 @@
         <v>2224.9499999999998</v>
       </c>
     </row>
-    <row r="99" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="99" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A99" t="s">
         <v>300</v>
       </c>
@@ -4486,7 +4502,7 @@
         <v>2092.38</v>
       </c>
     </row>
-    <row r="100" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="100" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A100" t="s">
         <v>302</v>
       </c>
@@ -4500,7 +4516,7 @@
         <v>1324.1</v>
       </c>
     </row>
-    <row r="101" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="101" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A101" t="s">
         <v>304</v>
       </c>
@@ -4514,7 +4530,7 @@
         <v>1278.25</v>
       </c>
     </row>
-    <row r="102" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="102" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A102" t="s">
         <v>306</v>
       </c>
@@ -4528,7 +4544,7 @@
         <v>2082.62</v>
       </c>
     </row>
-    <row r="103" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="103" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A103" t="s">
         <v>308</v>
       </c>
@@ -4542,7 +4558,7 @@
         <v>1288.21</v>
       </c>
     </row>
-    <row r="104" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="104" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A104" t="s">
         <v>310</v>
       </c>
@@ -4556,7 +4572,7 @@
         <v>1286.55</v>
       </c>
     </row>
-    <row r="105" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="105" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A105" t="s">
         <v>312</v>
       </c>
@@ -4570,7 +4586,7 @@
         <v>1988.43</v>
       </c>
     </row>
-    <row r="106" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="106" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A106" t="s">
         <v>314</v>
       </c>
@@ -4584,7 +4600,7 @@
         <v>1285.0899999999999</v>
       </c>
     </row>
-    <row r="107" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="107" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A107" t="s">
         <v>316</v>
       </c>
@@ -4598,7 +4614,7 @@
         <v>5223.16</v>
       </c>
     </row>
-    <row r="108" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="108" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A108" t="s">
         <v>318</v>
       </c>
@@ -4612,7 +4628,7 @@
         <v>5346.6</v>
       </c>
     </row>
-    <row r="109" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="109" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A109" t="s">
         <v>320</v>
       </c>
@@ -4626,7 +4642,7 @@
         <v>6451.4</v>
       </c>
     </row>
-    <row r="110" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="110" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A110" t="s">
         <v>322</v>
       </c>
@@ -4640,7 +4656,7 @@
         <v>181867.97</v>
       </c>
     </row>
-    <row r="111" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="111" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A111" t="s">
         <v>324</v>
       </c>
@@ -4654,7 +4670,7 @@
         <v>1401.49</v>
       </c>
     </row>
-    <row r="112" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="112" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A112" t="s">
         <v>326</v>
       </c>
@@ -4668,7 +4684,7 @@
         <v>1409.37</v>
       </c>
     </row>
-    <row r="113" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="113" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A113" t="s">
         <v>328</v>
       </c>
@@ -4682,7 +4698,7 @@
         <v>1399.62</v>
       </c>
     </row>
-    <row r="114" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="114" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A114" t="s">
         <v>329</v>
       </c>
@@ -4696,7 +4712,7 @@
         <v>5223.16</v>
       </c>
     </row>
-    <row r="115" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="115" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A115" t="s">
         <v>331</v>
       </c>
@@ -4710,7 +4726,7 @@
         <v>5346.6</v>
       </c>
     </row>
-    <row r="116" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="116" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A116" t="s">
         <v>333</v>
       </c>
@@ -4724,7 +4740,7 @@
         <v>1824.32</v>
       </c>
     </row>
-    <row r="117" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="117" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A117" t="s">
         <v>335</v>
       </c>
@@ -4738,7 +4754,7 @@
         <v>6451.4</v>
       </c>
     </row>
-    <row r="118" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="118" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A118" t="s">
         <v>337</v>
       </c>
@@ -4752,7 +4768,7 @@
         <v>6453.69</v>
       </c>
     </row>
-    <row r="119" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="119" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A119" t="s">
         <v>339</v>
       </c>
@@ -4766,7 +4782,7 @@
         <v>1401.28</v>
       </c>
     </row>
-    <row r="120" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="120" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A120" t="s">
         <v>341</v>
       </c>
@@ -4780,7 +4796,7 @@
         <v>1568.92</v>
       </c>
     </row>
-    <row r="121" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="121" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A121" t="s">
         <v>343</v>
       </c>
@@ -4794,7 +4810,7 @@
         <v>5328.35</v>
       </c>
     </row>
-    <row r="122" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="122" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A122" t="s">
         <v>345</v>
       </c>
@@ -4808,7 +4824,7 @@
         <v>5451.59</v>
       </c>
     </row>
-    <row r="123" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="123" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A123" t="s">
         <v>347</v>
       </c>
@@ -4822,7 +4838,7 @@
         <v>1836.77</v>
       </c>
     </row>
-    <row r="124" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="124" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A124" t="s">
         <v>349</v>
       </c>
@@ -4836,7 +4852,7 @@
         <v>6556.18</v>
       </c>
     </row>
-    <row r="125" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="125" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A125" t="s">
         <v>351</v>
       </c>
@@ -4850,7 +4866,7 @@
         <v>6558.46</v>
       </c>
     </row>
-    <row r="126" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="126" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A126" t="s">
         <v>353</v>
       </c>
@@ -4864,7 +4880,7 @@
         <v>1606.89</v>
       </c>
     </row>
-    <row r="127" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="127" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A127" t="s">
         <v>355</v>
       </c>
@@ -4878,7 +4894,7 @@
         <v>1629.71</v>
       </c>
     </row>
-    <row r="128" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="128" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A128" t="s">
         <v>357</v>
       </c>
@@ -4892,7 +4908,7 @@
         <v>1627.84</v>
       </c>
     </row>
-    <row r="129" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="129" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A129" t="s">
         <v>359</v>
       </c>
@@ -4906,7 +4922,7 @@
         <v>5387.06</v>
       </c>
     </row>
-    <row r="130" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="130" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A130" t="s">
         <v>361</v>
       </c>
@@ -4920,7 +4936,7 @@
         <v>5510.72</v>
       </c>
     </row>
-    <row r="131" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="131" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A131" t="s">
         <v>363</v>
       </c>
@@ -4934,7 +4950,7 @@
         <v>6615.31</v>
       </c>
     </row>
-    <row r="132" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="132" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A132" t="s">
         <v>365</v>
       </c>
@@ -4948,7 +4964,7 @@
         <v>6617.38</v>
       </c>
     </row>
-    <row r="133" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="133" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A133" t="s">
         <v>367</v>
       </c>
@@ -4962,7 +4978,7 @@
         <v>1771.62</v>
       </c>
     </row>
-    <row r="134" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="134" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A134" t="s">
         <v>418</v>
       </c>
@@ -4976,7 +4992,7 @@
         <v>4350.1099999999997</v>
       </c>
     </row>
-    <row r="135" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="135" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A135" t="s">
         <v>420</v>
       </c>
@@ -4990,7 +5006,7 @@
         <v>4274.79</v>
       </c>
     </row>
-    <row r="136" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="136" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A136" t="s">
         <v>422</v>
       </c>
@@ -5004,7 +5020,7 @@
         <v>4233.71</v>
       </c>
     </row>
-    <row r="137" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="137" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A137" t="s">
         <v>424</v>
       </c>
@@ -5018,7 +5034,7 @@
         <v>4150.3100000000004</v>
       </c>
     </row>
-    <row r="138" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="138" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A138" t="s">
         <v>426</v>
       </c>
@@ -5032,7 +5048,7 @@
         <v>4150.3100000000004</v>
       </c>
     </row>
-    <row r="139" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="139" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A139" t="s">
         <v>428</v>
       </c>
@@ -5046,7 +5062,7 @@
         <v>4055.29</v>
       </c>
     </row>
-    <row r="140" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="140" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A140" t="s">
         <v>430</v>
       </c>
@@ -5060,7 +5076,7 @@
         <v>4345.75</v>
       </c>
     </row>
-    <row r="141" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="141" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A141" t="s">
         <v>432</v>
       </c>
@@ -5074,7 +5090,7 @@
         <v>8853.39</v>
       </c>
     </row>
-    <row r="142" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="142" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A142" t="s">
         <v>434</v>
       </c>
@@ -5088,7 +5104,7 @@
         <v>5884.59</v>
       </c>
     </row>
-    <row r="143" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="143" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A143" t="s">
         <v>436</v>
       </c>
@@ -5102,7 +5118,7 @@
         <v>4350.1099999999997</v>
       </c>
     </row>
-    <row r="144" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="144" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A144" t="s">
         <v>438</v>
       </c>
@@ -5116,7 +5132,7 @@
         <v>4274.79</v>
       </c>
     </row>
-    <row r="145" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="145" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A145" t="s">
         <v>440</v>
       </c>
@@ -5130,7 +5146,7 @@
         <v>4233.71</v>
       </c>
     </row>
-    <row r="146" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="146" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A146" t="s">
         <v>442</v>
       </c>
@@ -5144,7 +5160,7 @@
         <v>7950.61</v>
       </c>
     </row>
-    <row r="147" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="147" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A147" t="s">
         <v>444</v>
       </c>
@@ -5158,7 +5174,7 @@
         <v>8070.74</v>
       </c>
     </row>
-    <row r="148" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="148" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A148" t="s">
         <v>446</v>
       </c>
@@ -5172,7 +5188,7 @@
         <v>4150.3100000000004</v>
       </c>
     </row>
-    <row r="149" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="149" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A149" t="s">
         <v>448</v>
       </c>
@@ -5186,7 +5202,7 @@
         <v>4150.3100000000004</v>
       </c>
     </row>
-    <row r="150" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="150" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A150" t="s">
         <v>450</v>
       </c>
@@ -5200,7 +5216,7 @@
         <v>4055.29</v>
       </c>
     </row>
-    <row r="151" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="151" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A151" t="s">
         <v>452</v>
       </c>
@@ -5214,7 +5230,7 @@
         <v>8447.1</v>
       </c>
     </row>
-    <row r="152" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="152" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A152" t="s">
         <v>454</v>
       </c>
@@ -5228,7 +5244,7 @@
         <v>8567.2199999999993</v>
       </c>
     </row>
-    <row r="153" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="153" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A153" t="s">
         <v>475</v>
       </c>
@@ -5242,7 +5258,7 @@
         <v>9216.2000000000007</v>
       </c>
     </row>
-    <row r="154" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="154" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A154" t="s">
         <v>477</v>
       </c>
@@ -5256,7 +5272,7 @@
         <v>9243.7999999999993</v>
       </c>
     </row>
-    <row r="155" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="155" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A155" t="s">
         <v>479</v>
       </c>
@@ -5270,7 +5286,7 @@
         <v>4345.75</v>
       </c>
     </row>
-    <row r="156" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="156" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A156" t="s">
         <v>481</v>
       </c>
@@ -5284,7 +5300,7 @@
         <v>6026.7</v>
       </c>
     </row>
-    <row r="157" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="157" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A157" t="s">
         <v>483</v>
       </c>
@@ -5298,7 +5314,7 @@
         <v>9820.7800000000007</v>
       </c>
     </row>
-    <row r="158" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="158" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A158" t="s">
         <v>485</v>
       </c>
@@ -5312,7 +5328,7 @@
         <v>10029.5</v>
       </c>
     </row>
-    <row r="159" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="159" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A159" t="s">
         <v>487</v>
       </c>
@@ -5326,7 +5342,7 @@
         <v>5884.59</v>
       </c>
     </row>
-    <row r="160" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="160" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A160" t="s">
         <v>489</v>
       </c>
@@ -5340,7 +5356,7 @@
         <v>4350.1099999999997</v>
       </c>
     </row>
-    <row r="161" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="161" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A161" t="s">
         <v>491</v>
       </c>
@@ -5354,7 +5370,7 @@
         <v>4274.79</v>
       </c>
     </row>
-    <row r="162" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="162" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A162" t="s">
         <v>493</v>
       </c>
@@ -5368,7 +5384,7 @@
         <v>4233.71</v>
       </c>
     </row>
-    <row r="163" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="163" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A163" t="s">
         <v>495</v>
       </c>
@@ -5382,7 +5398,7 @@
         <v>3840.14</v>
       </c>
     </row>
-    <row r="164" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="164" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A164" t="s">
         <v>497</v>
       </c>
@@ -5396,7 +5412,7 @@
         <v>8719.51</v>
       </c>
     </row>
-    <row r="165" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="165" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A165" t="s">
         <v>499</v>
       </c>
@@ -5410,7 +5426,7 @@
         <v>4150.3100000000004</v>
       </c>
     </row>
-    <row r="166" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="166" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A166" t="s">
         <v>501</v>
       </c>
@@ -5424,7 +5440,7 @@
         <v>4150.3100000000004</v>
       </c>
     </row>
-    <row r="167" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="167" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A167" t="s">
         <v>503</v>
       </c>
@@ -5438,7 +5454,7 @@
         <v>4055.29</v>
       </c>
     </row>
-    <row r="168" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="168" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A168" t="s">
         <v>505</v>
       </c>
@@ -5452,7 +5468,7 @@
         <v>8447.1</v>
       </c>
     </row>
-    <row r="169" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="169" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A169" t="s">
         <v>507</v>
       </c>
@@ -5466,7 +5482,7 @@
         <v>8567.2199999999993</v>
       </c>
     </row>
-    <row r="170" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="170" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A170" t="s">
         <v>509</v>
       </c>
@@ -5480,7 +5496,7 @@
         <v>8205.39</v>
       </c>
     </row>
-    <row r="171" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="171" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A171" t="s">
         <v>510</v>
       </c>
@@ -5494,7 +5510,7 @@
         <v>4248.24</v>
       </c>
     </row>
-    <row r="172" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="172" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A172" t="s">
         <v>512</v>
       </c>
@@ -5508,7 +5524,7 @@
         <v>9216.2000000000007</v>
       </c>
     </row>
-    <row r="173" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="173" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A173" t="s">
         <v>514</v>
       </c>
@@ -5522,7 +5538,7 @@
         <v>9243.7999999999993</v>
       </c>
     </row>
-    <row r="174" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="174" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A174" t="s">
         <v>516</v>
       </c>
@@ -5536,7 +5552,7 @@
         <v>9354.7999999999993</v>
       </c>
     </row>
-    <row r="175" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="175" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A175" t="s">
         <v>518</v>
       </c>
@@ -5550,7 +5566,7 @@
         <v>4345.75</v>
       </c>
     </row>
-    <row r="176" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="176" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A176" t="s">
         <v>520</v>
       </c>
@@ -5564,7 +5580,7 @@
         <v>6026.7</v>
       </c>
     </row>
-    <row r="177" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="177" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A177" t="s">
         <v>522</v>
       </c>
@@ -5578,7 +5594,7 @@
         <v>9820.7800000000007</v>
       </c>
     </row>
-    <row r="178" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="178" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A178" t="s">
         <v>524</v>
       </c>
@@ -5592,7 +5608,7 @@
         <v>10055.64</v>
       </c>
     </row>
-    <row r="179" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="179" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A179" t="s">
         <v>526</v>
       </c>
@@ -5606,7 +5622,7 @@
         <v>5787.69</v>
       </c>
     </row>
-    <row r="180" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="180" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A180" t="s">
         <v>528</v>
       </c>
@@ -5620,7 +5636,7 @@
         <v>10818.52</v>
       </c>
     </row>
-    <row r="181" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="181" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A181" t="s">
         <v>530</v>
       </c>
@@ -5634,7 +5650,7 @@
         <v>10846.12</v>
       </c>
     </row>
-    <row r="182" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="182" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A182" t="s">
         <v>532</v>
       </c>
@@ -5648,7 +5664,7 @@
         <v>10857.32</v>
       </c>
     </row>
-    <row r="183" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="183" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A183" t="s">
         <v>534</v>
       </c>
@@ -5662,7 +5678,7 @@
         <v>5884.59</v>
       </c>
     </row>
-    <row r="184" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="184" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A184" t="s">
         <v>536</v>
       </c>
@@ -5676,7 +5692,7 @@
         <v>8246.0499999999993</v>
       </c>
     </row>
-    <row r="185" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="185" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A185" t="s">
         <v>538</v>
       </c>
@@ -5690,7 +5706,7 @@
         <v>8103.73</v>
       </c>
     </row>
-    <row r="186" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="186" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A186" t="s">
         <v>571</v>
       </c>
@@ -5704,7 +5720,7 @@
         <v>11861.29</v>
       </c>
     </row>
-    <row r="187" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="187" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A187" t="s">
         <v>573</v>
       </c>
@@ -5718,7 +5734,7 @@
         <v>11972.29</v>
       </c>
     </row>
-    <row r="188" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="188" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A188" t="s">
         <v>575</v>
       </c>
@@ -5732,7 +5748,7 @@
         <v>11967.52</v>
       </c>
     </row>
-    <row r="189" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="189" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A189" t="s">
         <v>577</v>
       </c>
@@ -5746,7 +5762,7 @@
         <v>9089.85</v>
       </c>
     </row>
-    <row r="190" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="190" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A190" t="s">
         <v>579</v>
       </c>
@@ -5760,7 +5776,7 @@
         <v>11282.44</v>
       </c>
     </row>
-    <row r="191" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="191" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A191" t="s">
         <v>581</v>
       </c>
@@ -5774,7 +5790,7 @@
         <v>11289.7</v>
       </c>
     </row>
-    <row r="192" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="192" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A192" t="s">
         <v>583</v>
       </c>
@@ -5788,7 +5804,7 @@
         <v>14412.18</v>
       </c>
     </row>
-    <row r="193" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="193" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A193" t="s">
         <v>585</v>
       </c>
@@ -5802,7 +5818,7 @@
         <v>11972.29</v>
       </c>
     </row>
-    <row r="194" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="194" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A194" t="s">
         <v>587</v>
       </c>
@@ -5816,7 +5832,7 @@
         <v>9344.2099999999991</v>
       </c>
     </row>
-    <row r="195" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="195" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A195" t="s">
         <v>589</v>
       </c>
@@ -5830,7 +5846,7 @@
         <v>11861.29</v>
       </c>
     </row>
-    <row r="196" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="196" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A196" t="s">
         <v>591</v>
       </c>
@@ -5844,7 +5860,7 @@
         <v>13086.63</v>
       </c>
     </row>
-    <row r="197" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="197" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A197" t="s">
         <v>593</v>
       </c>
@@ -5858,7 +5874,7 @@
         <v>11289.7</v>
       </c>
     </row>
-    <row r="198" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="198" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A198" t="s">
         <v>595</v>
       </c>
@@ -5872,7 +5888,7 @@
         <v>14386.87</v>
       </c>
     </row>
-    <row r="199" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="199" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A199" t="s">
         <v>597</v>
       </c>
@@ -5886,7 +5902,7 @@
         <v>13169.62</v>
       </c>
     </row>
-    <row r="200" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="200" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A200" t="s">
         <v>613</v>
       </c>
@@ -5900,7 +5916,7 @@
         <v>21767.34</v>
       </c>
     </row>
-    <row r="201" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="201" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A201" t="s">
         <v>615</v>
       </c>
@@ -5914,7 +5930,7 @@
         <v>22062.37</v>
       </c>
     </row>
-    <row r="202" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="202" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A202" t="s">
         <v>617</v>
       </c>
@@ -5928,7 +5944,7 @@
         <v>21811.119999999999</v>
       </c>
     </row>
-    <row r="203" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="203" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A203" t="s">
         <v>619</v>
       </c>
@@ -5942,7 +5958,7 @@
         <v>23638.14</v>
       </c>
     </row>
-    <row r="204" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="204" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A204" t="s">
         <v>621</v>
       </c>
@@ -5956,7 +5972,7 @@
         <v>23807.02</v>
       </c>
     </row>
-    <row r="205" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="205" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A205" t="s">
         <v>623</v>
       </c>
@@ -5970,7 +5986,7 @@
         <v>23592.91</v>
       </c>
     </row>
-    <row r="206" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="206" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A206" t="s">
         <v>625</v>
       </c>
@@ -5984,7 +6000,7 @@
         <v>21767.34</v>
       </c>
     </row>
-    <row r="207" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="207" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A207" t="s">
         <v>627</v>
       </c>
@@ -5998,7 +6014,7 @@
         <v>22062.37</v>
       </c>
     </row>
-    <row r="208" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="208" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A208" t="s">
         <v>629</v>
       </c>
@@ -6012,7 +6028,7 @@
         <v>20351.330000000002</v>
       </c>
     </row>
-    <row r="209" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="209" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A209" t="s">
         <v>631</v>
       </c>
@@ -6026,7 +6042,7 @@
         <v>23496.22</v>
       </c>
     </row>
-    <row r="210" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="210" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A210" t="s">
         <v>632</v>
       </c>
@@ -6040,7 +6056,7 @@
         <v>26001.89</v>
       </c>
     </row>
-    <row r="211" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="211" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A211" t="s">
         <v>634</v>
       </c>
@@ -6054,7 +6070,7 @@
         <v>23807.02</v>
       </c>
     </row>
-    <row r="212" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="212" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A212" t="s">
         <v>636</v>
       </c>
@@ -6068,7 +6084,7 @@
         <v>23676.31</v>
       </c>
     </row>
-    <row r="213" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="213" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A213" t="s">
         <v>638</v>
       </c>
@@ -6082,7 +6098,7 @@
         <v>23621.54</v>
       </c>
     </row>
-    <row r="214" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="214" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A214" t="s">
         <v>639</v>
       </c>
@@ -6096,7 +6112,7 @@
         <v>23700.17</v>
       </c>
     </row>
-    <row r="215" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="215" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A215" t="s">
         <v>641</v>
       </c>
@@ -6110,7 +6126,7 @@
         <v>24183.79</v>
       </c>
     </row>
-    <row r="216" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="216" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A216" t="s">
         <v>659</v>
       </c>
@@ -6124,7 +6140,7 @@
         <v>38736.639999999999</v>
       </c>
     </row>
-    <row r="217" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="217" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A217" t="s">
         <v>661</v>
       </c>
@@ -6138,7 +6154,7 @@
         <v>38837.89</v>
       </c>
     </row>
-    <row r="218" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="218" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A218" t="s">
         <v>663</v>
       </c>
@@ -6152,7 +6168,7 @@
         <v>48561.36</v>
       </c>
     </row>
-    <row r="219" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="219" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A219" t="s">
         <v>665</v>
       </c>
@@ -6166,7 +6182,7 @@
         <v>40701</v>
       </c>
     </row>
-    <row r="220" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="220" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A220" t="s">
         <v>667</v>
       </c>
@@ -6180,7 +6196,7 @@
         <v>51251.47</v>
       </c>
     </row>
-    <row r="221" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="221" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A221" t="s">
         <v>669</v>
       </c>
@@ -6195,6 +6211,19 @@
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="A1:D221" xr:uid="{7946CC59-6F99-4531-BC40-6D94404CB3C2}">
+    <filterColumn colId="0">
+      <filters>
+        <filter val="PDG43M0800P2MN"/>
+        <filter val="PDG53K0800P2MN"/>
+        <filter val="PDG53K1200P2MN"/>
+        <filter val="PDG53M0800P2MN"/>
+        <filter val="PDG53M1200P2MN"/>
+        <filter val="PDG63M1600P2MN"/>
+        <filter val="PDG63M2000P2MN"/>
+      </filters>
+    </filterColumn>
+  </autoFilter>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>